<commit_message>
Add role-based login screen for Customer/Vendor/Admin, dedicated Profile screen, and top back navigation buttons across all views
</commit_message>
<xml_diff>
--- a/SpotCart_Selenium_E2E_Test_Report.xlsx
+++ b/SpotCart_Selenium_E2E_Test_Report.xlsx
@@ -565,7 +565,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-07-28 08:53:49 IST</t>
+          <t>2026-07-28 09:07:05 IST</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="F2" s="9" t="n">
-        <v>1.776</v>
+        <v>1.603</v>
       </c>
       <c r="G2" s="12" t="inlineStr">
         <is>
@@ -1027,7 +1027,7 @@
         </is>
       </c>
       <c r="F3" s="9" t="n">
-        <v>1.037</v>
+        <v>0.523</v>
       </c>
       <c r="G3" s="12" t="inlineStr">
         <is>
@@ -1067,7 +1067,7 @@
         </is>
       </c>
       <c r="F4" s="9" t="n">
-        <v>0.011</v>
+        <v>0.016</v>
       </c>
       <c r="G4" s="12" t="inlineStr">
         <is>
@@ -1107,7 +1107,7 @@
         </is>
       </c>
       <c r="F5" s="9" t="n">
-        <v>0.013</v>
+        <v>0.015</v>
       </c>
       <c r="G5" s="12" t="inlineStr">
         <is>
@@ -1227,7 +1227,7 @@
         </is>
       </c>
       <c r="F8" s="9" t="n">
-        <v>1.011</v>
+        <v>1.014</v>
       </c>
       <c r="G8" s="12" t="inlineStr">
         <is>
@@ -1267,7 +1267,7 @@
         </is>
       </c>
       <c r="F9" s="9" t="n">
-        <v>1.062</v>
+        <v>1.069</v>
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
@@ -1316,7 +1316,7 @@
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>Total Page Load: 746ms, DOM Interactive: 746ms</t>
+          <t>Total Page Load: 579ms, DOM Interactive: 579ms</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update profile screen & OTP registration with real Name, Phone, User ID/Email, Password/PIN fields and live edit bottom sheet
</commit_message>
<xml_diff>
--- a/SpotCart_Selenium_E2E_Test_Report.xlsx
+++ b/SpotCart_Selenium_E2E_Test_Report.xlsx
@@ -565,7 +565,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-07-28 09:07:05 IST</t>
+          <t>2026-07-28 09:12:13 IST</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="F2" s="9" t="n">
-        <v>1.603</v>
+        <v>1.778</v>
       </c>
       <c r="G2" s="12" t="inlineStr">
         <is>
@@ -1027,7 +1027,7 @@
         </is>
       </c>
       <c r="F3" s="9" t="n">
-        <v>0.523</v>
+        <v>0.554</v>
       </c>
       <c r="G3" s="12" t="inlineStr">
         <is>
@@ -1067,7 +1067,7 @@
         </is>
       </c>
       <c r="F4" s="9" t="n">
-        <v>0.016</v>
+        <v>0.011</v>
       </c>
       <c r="G4" s="12" t="inlineStr">
         <is>
@@ -1107,7 +1107,7 @@
         </is>
       </c>
       <c r="F5" s="9" t="n">
-        <v>0.015</v>
+        <v>0.013</v>
       </c>
       <c r="G5" s="12" t="inlineStr">
         <is>
@@ -1147,7 +1147,7 @@
         </is>
       </c>
       <c r="F6" s="9" t="n">
-        <v>2.011</v>
+        <v>2.01</v>
       </c>
       <c r="G6" s="12" t="inlineStr">
         <is>
@@ -1227,7 +1227,7 @@
         </is>
       </c>
       <c r="F8" s="9" t="n">
-        <v>1.014</v>
+        <v>1.012</v>
       </c>
       <c r="G8" s="12" t="inlineStr">
         <is>
@@ -1267,7 +1267,7 @@
         </is>
       </c>
       <c r="F9" s="9" t="n">
-        <v>1.069</v>
+        <v>1.081</v>
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
@@ -1316,7 +1316,7 @@
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>Total Page Load: 579ms, DOM Interactive: 579ms</t>
+          <t>Total Page Load: 756ms, DOM Interactive: 756ms</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Make phone OTP verification & Firestore user session creation 100% resilient across Web and Mobile
</commit_message>
<xml_diff>
--- a/SpotCart_Selenium_E2E_Test_Report.xlsx
+++ b/SpotCart_Selenium_E2E_Test_Report.xlsx
@@ -565,7 +565,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-07-28 09:12:13 IST</t>
+          <t>2026-07-28 09:20:10 IST</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="F2" s="9" t="n">
-        <v>1.778</v>
+        <v>1.614</v>
       </c>
       <c r="G2" s="12" t="inlineStr">
         <is>
@@ -1027,7 +1027,7 @@
         </is>
       </c>
       <c r="F3" s="9" t="n">
-        <v>0.554</v>
+        <v>0.006</v>
       </c>
       <c r="G3" s="12" t="inlineStr">
         <is>
@@ -1067,7 +1067,7 @@
         </is>
       </c>
       <c r="F4" s="9" t="n">
-        <v>0.011</v>
+        <v>0.01</v>
       </c>
       <c r="G4" s="12" t="inlineStr">
         <is>
@@ -1107,7 +1107,7 @@
         </is>
       </c>
       <c r="F5" s="9" t="n">
-        <v>0.013</v>
+        <v>0.014</v>
       </c>
       <c r="G5" s="12" t="inlineStr">
         <is>
@@ -1267,7 +1267,7 @@
         </is>
       </c>
       <c r="F9" s="9" t="n">
-        <v>1.081</v>
+        <v>1.064</v>
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
@@ -1316,7 +1316,7 @@
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>Total Page Load: 756ms, DOM Interactive: 756ms</t>
+          <t>Total Page Load: 594ms, DOM Interactive: 594ms</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add reCAPTCHA container for Web SMS Auth and enhance phone formatting with SMS notification
</commit_message>
<xml_diff>
--- a/SpotCart_Selenium_E2E_Test_Report.xlsx
+++ b/SpotCart_Selenium_E2E_Test_Report.xlsx
@@ -565,7 +565,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-07-28 09:20:10 IST</t>
+          <t>2026-07-28 09:27:45 IST</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="F2" s="9" t="n">
-        <v>1.614</v>
+        <v>1.713</v>
       </c>
       <c r="G2" s="12" t="inlineStr">
         <is>
@@ -1027,7 +1027,7 @@
         </is>
       </c>
       <c r="F3" s="9" t="n">
-        <v>0.006</v>
+        <v>0.007</v>
       </c>
       <c r="G3" s="12" t="inlineStr">
         <is>
@@ -1067,7 +1067,7 @@
         </is>
       </c>
       <c r="F4" s="9" t="n">
-        <v>0.01</v>
+        <v>0.023</v>
       </c>
       <c r="G4" s="12" t="inlineStr">
         <is>
@@ -1107,7 +1107,7 @@
         </is>
       </c>
       <c r="F5" s="9" t="n">
-        <v>0.014</v>
+        <v>0.058</v>
       </c>
       <c r="G5" s="12" t="inlineStr">
         <is>
@@ -1227,7 +1227,7 @@
         </is>
       </c>
       <c r="F8" s="9" t="n">
-        <v>1.012</v>
+        <v>1.014</v>
       </c>
       <c r="G8" s="12" t="inlineStr">
         <is>
@@ -1267,7 +1267,7 @@
         </is>
       </c>
       <c r="F9" s="9" t="n">
-        <v>1.064</v>
+        <v>1.066</v>
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
@@ -1316,7 +1316,7 @@
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>Total Page Load: 594ms, DOM Interactive: 594ms</t>
+          <t>Total Page Load: 695ms, DOM Interactive: 695ms</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Admin Support & Query Resolution Center for customer/vendor queries and start app on Login Screen
</commit_message>
<xml_diff>
--- a/SpotCart_Selenium_E2E_Test_Report.xlsx
+++ b/SpotCart_Selenium_E2E_Test_Report.xlsx
@@ -565,7 +565,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-07-28 09:27:45 IST</t>
+          <t>2026-07-28 11:38:48 IST</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="F2" s="9" t="n">
-        <v>1.713</v>
+        <v>1.601</v>
       </c>
       <c r="G2" s="12" t="inlineStr">
         <is>
@@ -1027,7 +1027,7 @@
         </is>
       </c>
       <c r="F3" s="9" t="n">
-        <v>0.007</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="G3" s="12" t="inlineStr">
         <is>
@@ -1067,7 +1067,7 @@
         </is>
       </c>
       <c r="F4" s="9" t="n">
-        <v>0.023</v>
+        <v>0.051</v>
       </c>
       <c r="G4" s="12" t="inlineStr">
         <is>
@@ -1107,7 +1107,7 @@
         </is>
       </c>
       <c r="F5" s="9" t="n">
-        <v>0.058</v>
+        <v>0.094</v>
       </c>
       <c r="G5" s="12" t="inlineStr">
         <is>
@@ -1147,7 +1147,7 @@
         </is>
       </c>
       <c r="F6" s="9" t="n">
-        <v>2.01</v>
+        <v>2.011</v>
       </c>
       <c r="G6" s="12" t="inlineStr">
         <is>
@@ -1227,7 +1227,7 @@
         </is>
       </c>
       <c r="F8" s="9" t="n">
-        <v>1.014</v>
+        <v>1.011</v>
       </c>
       <c r="G8" s="12" t="inlineStr">
         <is>
@@ -1267,7 +1267,7 @@
         </is>
       </c>
       <c r="F9" s="9" t="n">
-        <v>1.066</v>
+        <v>1.047</v>
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
@@ -1307,7 +1307,7 @@
         </is>
       </c>
       <c r="F10" s="9" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G10" s="12" t="inlineStr">
         <is>
@@ -1316,7 +1316,7 @@
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>Total Page Load: 695ms, DOM Interactive: 695ms</t>
+          <t>Total Page Load: 573ms, DOM Interactive: 573ms</t>
         </is>
       </c>
     </row>
@@ -1347,7 +1347,7 @@
         </is>
       </c>
       <c r="F11" s="9" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G11" s="12" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add Appium Mobile E2E test suite, test datasets, and excel report in Mobile App appium testing folder with 10/10 PASS
</commit_message>
<xml_diff>
--- a/SpotCart_Selenium_E2E_Test_Report.xlsx
+++ b/SpotCart_Selenium_E2E_Test_Report.xlsx
@@ -565,7 +565,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-07-28 11:38:48 IST</t>
+          <t>2026-07-28 14:09:23 IST</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="F2" s="9" t="n">
-        <v>1.601</v>
+        <v>2.137</v>
       </c>
       <c r="G2" s="12" t="inlineStr">
         <is>
@@ -1027,7 +1027,7 @@
         </is>
       </c>
       <c r="F3" s="9" t="n">
-        <v>0.008999999999999999</v>
+        <v>3.094</v>
       </c>
       <c r="G3" s="12" t="inlineStr">
         <is>
@@ -1067,7 +1067,7 @@
         </is>
       </c>
       <c r="F4" s="9" t="n">
-        <v>0.051</v>
+        <v>0.018</v>
       </c>
       <c r="G4" s="12" t="inlineStr">
         <is>
@@ -1107,7 +1107,7 @@
         </is>
       </c>
       <c r="F5" s="9" t="n">
-        <v>0.094</v>
+        <v>0.018</v>
       </c>
       <c r="G5" s="12" t="inlineStr">
         <is>
@@ -1147,7 +1147,7 @@
         </is>
       </c>
       <c r="F6" s="9" t="n">
-        <v>2.011</v>
+        <v>2.007</v>
       </c>
       <c r="G6" s="12" t="inlineStr">
         <is>
@@ -1187,7 +1187,7 @@
         </is>
       </c>
       <c r="F7" s="9" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G7" s="12" t="inlineStr">
         <is>
@@ -1227,7 +1227,7 @@
         </is>
       </c>
       <c r="F8" s="9" t="n">
-        <v>1.011</v>
+        <v>1.01</v>
       </c>
       <c r="G8" s="12" t="inlineStr">
         <is>
@@ -1267,7 +1267,7 @@
         </is>
       </c>
       <c r="F9" s="9" t="n">
-        <v>1.047</v>
+        <v>1.051</v>
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
@@ -1316,7 +1316,7 @@
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>Total Page Load: 573ms, DOM Interactive: 573ms</t>
+          <t>Total Page Load: 1115ms, DOM Interactive: 1114ms</t>
         </is>
       </c>
     </row>

</xml_diff>